<commit_message>
update: add earnings + conversion block below donut chart in Deals sheet
</commit_message>
<xml_diff>
--- a/liberty-leads-v5.xlsx
+++ b/liberty-leads-v5.xlsx
@@ -20,11 +20,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="DD.MM.YY"/>
     <numFmt numFmtId="165" formatCode="#,##0 &quot;грн&quot;"/>
+    <numFmt numFmtId="166" formatCode="0.0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="37">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -169,6 +170,62 @@
       <b val="1"/>
       <color rgb="00D97706"/>
       <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00064E3B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00059669"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001D4ED8"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00065F46"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E40AF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="0092400E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+      <sz val="18"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -321,7 +378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -460,6 +517,39 @@
     <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="27" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="28" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="31" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="32" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="34" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -478,38 +568,38 @@
     <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -32037,7 +32127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J110"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -32047,8 +32137,10 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="5" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="5" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
@@ -32342,7 +32434,7 @@
       <c r="E20" s="46" t="n"/>
       <c r="F20" s="47" t="n"/>
     </row>
-    <row r="21" ht="24" customHeight="1">
+    <row r="21" ht="28" customHeight="1">
       <c r="A21" s="36" t="n"/>
       <c r="B21" s="37">
         <f>IF(A21="","",IFERROR(INDEX('🗂 CRM База'!$B$3:$B$977,A21),"❓ Не знайдено"))</f>
@@ -32352,8 +32444,13 @@
       <c r="D21" s="39" t="n"/>
       <c r="E21" s="40" t="n"/>
       <c r="F21" s="41" t="n"/>
-    </row>
-    <row r="22" ht="24" customHeight="1">
+      <c r="I21" s="48" t="inlineStr">
+        <is>
+          <t>💰  ФІНАНСОВИЙ ПІДСУМОК</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
       <c r="A22" s="42" t="n"/>
       <c r="B22" s="43">
         <f>IF(A22="","",IFERROR(INDEX('🗂 CRM База'!$B$3:$B$977,A22),"❓ Не знайдено"))</f>
@@ -32363,8 +32460,17 @@
       <c r="D22" s="45" t="n"/>
       <c r="E22" s="46" t="n"/>
       <c r="F22" s="47" t="n"/>
-    </row>
-    <row r="23" ht="24" customHeight="1">
+      <c r="I22" s="49" t="inlineStr">
+        <is>
+          <t>Загальна виручка</t>
+        </is>
+      </c>
+      <c r="K22" s="50">
+        <f>SUMIF($C$3:$C$102,"Оплачено ✅",$D$3:$D$102)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
       <c r="A23" s="36" t="n"/>
       <c r="B23" s="37">
         <f>IF(A23="","",IFERROR(INDEX('🗂 CRM База'!$B$3:$B$977,A23),"❓ Не знайдено"))</f>
@@ -32374,8 +32480,17 @@
       <c r="D23" s="39" t="n"/>
       <c r="E23" s="40" t="n"/>
       <c r="F23" s="41" t="n"/>
-    </row>
-    <row r="24" ht="24" customHeight="1">
+      <c r="I23" s="49" t="inlineStr">
+        <is>
+          <t>Середній чек</t>
+        </is>
+      </c>
+      <c r="K23" s="51">
+        <f>IFERROR(SUMIF($C$3:$C$102,"Оплачено ✅",$D$3:$D$102)/COUNTIF($C$3:$C$102,"Оплачено ✅"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="8" customHeight="1">
       <c r="A24" s="42" t="n"/>
       <c r="B24" s="43">
         <f>IF(A24="","",IFERROR(INDEX('🗂 CRM База'!$B$3:$B$977,A24),"❓ Не знайдено"))</f>
@@ -32386,7 +32501,7 @@
       <c r="E24" s="46" t="n"/>
       <c r="F24" s="47" t="n"/>
     </row>
-    <row r="25" ht="24" customHeight="1">
+    <row r="25" ht="28" customHeight="1">
       <c r="A25" s="36" t="n"/>
       <c r="B25" s="37">
         <f>IF(A25="","",IFERROR(INDEX('🗂 CRM База'!$B$3:$B$977,A25),"❓ Не знайдено"))</f>
@@ -32396,8 +32511,13 @@
       <c r="D25" s="39" t="n"/>
       <c r="E25" s="40" t="n"/>
       <c r="F25" s="41" t="n"/>
-    </row>
-    <row r="26" ht="24" customHeight="1">
+      <c r="I25" s="52" t="inlineStr">
+        <is>
+          <t>📊  КОНВЕРСІЯ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
       <c r="A26" s="42" t="n"/>
       <c r="B26" s="43">
         <f>IF(A26="","",IFERROR(INDEX('🗂 CRM База'!$B$3:$B$977,A26),"❓ Не знайдено"))</f>
@@ -32407,8 +32527,18 @@
       <c r="D26" s="45" t="n"/>
       <c r="E26" s="46" t="n"/>
       <c r="F26" s="47" t="n"/>
-    </row>
-    <row r="27" ht="24" customHeight="1">
+      <c r="I26" s="53" t="inlineStr">
+        <is>
+          <t>Всього контактів</t>
+        </is>
+      </c>
+      <c r="K26" s="54" t="inlineStr">
+        <is>
+          <t>Оплачено</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
       <c r="A27" s="36" t="n"/>
       <c r="B27" s="37">
         <f>IF(A27="","",IFERROR(INDEX('🗂 CRM База'!$B$3:$B$977,A27),"❓ Не знайдено"))</f>
@@ -32418,8 +32548,16 @@
       <c r="D27" s="39" t="n"/>
       <c r="E27" s="40" t="n"/>
       <c r="F27" s="41" t="n"/>
-    </row>
-    <row r="28" ht="24" customHeight="1">
+      <c r="I27" s="55">
+        <f>COUNTA($A$3:$A$102)</f>
+        <v/>
+      </c>
+      <c r="K27" s="56">
+        <f>COUNTIF($C$3:$C$102,"Оплачено ✅")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
       <c r="A28" s="42" t="n"/>
       <c r="B28" s="43">
         <f>IF(A28="","",IFERROR(INDEX('🗂 CRM База'!$B$3:$B$977,A28),"❓ Не знайдено"))</f>
@@ -32429,6 +32567,15 @@
       <c r="D28" s="45" t="n"/>
       <c r="E28" s="46" t="n"/>
       <c r="F28" s="47" t="n"/>
+      <c r="I28" s="57" t="inlineStr">
+        <is>
+          <t>Конверсія в оплату</t>
+        </is>
+      </c>
+      <c r="K28" s="58">
+        <f>IFERROR(COUNTIF($C$3:$C$102,"Оплачено ✅")/COUNTA($A$3:$A$102)*100,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="36" t="n"/>
@@ -33245,13 +33392,13 @@
       <c r="F102" s="47" t="n"/>
     </row>
     <row r="104" ht="20" customHeight="1">
-      <c r="A104" s="48" t="inlineStr">
+      <c r="A104" s="59" t="inlineStr">
         <is>
           <t>💵 ЗАГАЛЬНА
 ВИРУЧКА</t>
         </is>
       </c>
-      <c r="C104" s="49">
+      <c r="C104" s="60">
         <f>SUMIF(C3:C102,"Оплачено ✅",D3:D102)</f>
         <v/>
       </c>
@@ -33260,39 +33407,51 @@
     <row r="106" ht="20" customHeight="1"/>
     <row r="107" ht="20" customHeight="1"/>
     <row r="109" ht="20" customHeight="1">
-      <c r="E109" s="50" t="inlineStr">
+      <c r="E109" s="61" t="inlineStr">
         <is>
           <t>Всього угод</t>
         </is>
       </c>
-      <c r="F109" s="50" t="inlineStr">
+      <c r="F109" s="61" t="inlineStr">
         <is>
           <t>Оплачено</t>
         </is>
       </c>
-      <c r="G109" s="50" t="inlineStr">
+      <c r="G109" s="61" t="inlineStr">
         <is>
           <t>Конверсія</t>
         </is>
       </c>
     </row>
     <row r="110" ht="32" customHeight="1">
-      <c r="E110" s="51">
+      <c r="E110" s="62">
         <f>COUNTA(A3:A102)</f>
         <v/>
       </c>
-      <c r="F110" s="52">
+      <c r="F110" s="63">
         <f>COUNTIF(C3:C102,"Оплачено ✅")</f>
         <v/>
       </c>
-      <c r="G110" s="53">
+      <c r="G110" s="64">
         <f>IFERROR(TEXT(COUNTIF(C3:C102,"Оплачено ✅")/COUNTA(A3:A102)*100,"0.0")&amp;"%","0%")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="15">
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="I25:L25"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="I21:L21"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="I26:J26"/>
     <mergeCell ref="C104:D107"/>
     <mergeCell ref="A104:B107"/>
   </mergeCells>
@@ -33640,63 +33799,63 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="B1" s="54" t="inlineStr">
+      <c r="B1" s="65" t="inlineStr">
         <is>
           <t>📖  ЛЕГЕНДА — ЛАНЦЮГ, СТАТУСИ, СКРИПТИ</t>
         </is>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="B2" s="55" t="inlineStr">
+      <c r="B2" s="66" t="inlineStr">
         <is>
           <t>⚡ ЯК ПРАЦЮЄ АВТО-ЛАНЦЮГ</t>
         </is>
       </c>
-      <c r="C2" s="56" t="n"/>
+      <c r="C2" s="67" t="n"/>
     </row>
     <row r="3" ht="26" customHeight="1">
-      <c r="B3" s="57" t="inlineStr">
+      <c r="B3" s="68" t="inlineStr">
         <is>
           <t>Введи/видали Website →</t>
         </is>
       </c>
-      <c r="C3" s="57" t="inlineStr">
+      <c r="C3" s="68" t="inlineStr">
         <is>
           <t>Колонка САЙТ автоматично стає ✅ або ❌</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="B4" s="57" t="inlineStr">
+      <c r="B4" s="68" t="inlineStr">
         <is>
           <t>Введи/видали Instagram →</t>
         </is>
       </c>
-      <c r="C4" s="57" t="inlineStr">
+      <c r="C4" s="68" t="inlineStr">
         <is>
           <t>Колонка IG автоматично стає ✅ або ❌</t>
         </is>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1">
-      <c r="B5" s="57" t="inlineStr">
+      <c r="B5" s="68" t="inlineStr">
         <is>
           <t>САЙТ + IG змінились →</t>
         </is>
       </c>
-      <c r="C5" s="57" t="inlineStr">
+      <c r="C5" s="68" t="inlineStr">
         <is>
           <t>ТИП ЛІДУ, ПРІОРИТЕТ, ПРИЧИНА, ПІДХІД — оновлюються самі</t>
         </is>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1">
-      <c r="B6" s="57" t="inlineStr">
+      <c r="B6" s="68" t="inlineStr">
         <is>
           <t>Уточнити ПРИЧИНУ/ПІДХІД →</t>
         </is>
       </c>
-      <c r="C6" s="57" t="inlineStr">
+      <c r="C6" s="68" t="inlineStr">
         <is>
           <t>Просто напиши своє значення — або вибери з дропдауну</t>
         </is>
@@ -33704,80 +33863,80 @@
     </row>
     <row r="7" ht="8" customHeight="1"/>
     <row r="8" ht="26" customHeight="1">
-      <c r="B8" s="58" t="inlineStr">
+      <c r="B8" s="69" t="inlineStr">
         <is>
           <t>СТАТУСИ CRM</t>
         </is>
       </c>
-      <c r="C8" s="56" t="n"/>
+      <c r="C8" s="67" t="n"/>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="B9" s="59" t="inlineStr">
-        <is>
-          <t>🟡 Новий</t>
-        </is>
-      </c>
-      <c r="C9" s="59" t="inlineStr">
+      <c r="B9" s="70" t="inlineStr">
+        <is>
+          <t>🟡 Новий</t>
+        </is>
+      </c>
+      <c r="C9" s="70" t="inlineStr">
         <is>
           <t>Перший контакт ще не відбувся</t>
         </is>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
-      <c r="B10" s="59" t="inlineStr">
+      <c r="B10" s="70" t="inlineStr">
         <is>
           <t>🔵 Домовляємось</t>
         </is>
       </c>
-      <c r="C10" s="59" t="inlineStr">
+      <c r="C10" s="70" t="inlineStr">
         <is>
           <t>Ведемо перемовини</t>
         </is>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="59" t="inlineStr">
+      <c r="B11" s="70" t="inlineStr">
         <is>
           <t>🟣 Презентація</t>
         </is>
       </c>
-      <c r="C11" s="59" t="inlineStr">
+      <c r="C11" s="70" t="inlineStr">
         <is>
           <t>Показали демо — liberty-cafe.onrender.com</t>
         </is>
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
-      <c r="B12" s="59" t="inlineStr">
+      <c r="B12" s="70" t="inlineStr">
         <is>
           <t>🟠 Думає</t>
         </is>
       </c>
-      <c r="C12" s="59" t="inlineStr">
+      <c r="C12" s="70" t="inlineStr">
         <is>
           <t>Клієнт розглядає пропозицію</t>
         </is>
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
-      <c r="B13" s="59" t="inlineStr">
+      <c r="B13" s="70" t="inlineStr">
         <is>
           <t>🟢 Продано</t>
         </is>
       </c>
-      <c r="C13" s="59" t="inlineStr">
+      <c r="C13" s="70" t="inlineStr">
         <is>
           <t>✅ Угода закрита — вноси суму в аркуш «Угоди»</t>
         </is>
       </c>
     </row>
     <row r="14" ht="26" customHeight="1">
-      <c r="B14" s="59" t="inlineStr">
+      <c r="B14" s="70" t="inlineStr">
         <is>
           <t>🔴 Відмовився</t>
         </is>
       </c>
-      <c r="C14" s="59" t="inlineStr">
+      <c r="C14" s="70" t="inlineStr">
         <is>
           <t>Повернись через 3 місяці</t>
         </is>
@@ -33785,44 +33944,44 @@
     </row>
     <row r="15" ht="8" customHeight="1"/>
     <row r="16" ht="26" customHeight="1">
-      <c r="B16" s="60" t="inlineStr">
+      <c r="B16" s="71" t="inlineStr">
         <is>
           <t>ТИП ЛІДУ → СТРАТЕГІЯ</t>
         </is>
       </c>
-      <c r="C16" s="56" t="n"/>
+      <c r="C16" s="67" t="n"/>
     </row>
     <row r="17" ht="26" customHeight="1">
-      <c r="B17" s="61" t="inlineStr">
+      <c r="B17" s="72" t="inlineStr">
         <is>
           <t>🔥 Без сайту</t>
         </is>
       </c>
-      <c r="C17" s="61" t="inlineStr">
+      <c r="C17" s="72" t="inlineStr">
         <is>
           <t>Дзвінок або візит → «Знайшов вас, немає сайту, є 5 хв?»</t>
         </is>
       </c>
     </row>
     <row r="18" ht="26" customHeight="1">
-      <c r="B18" s="61" t="inlineStr">
+      <c r="B18" s="72" t="inlineStr">
         <is>
           <t>📸 Instagram тільки</t>
         </is>
       </c>
-      <c r="C18" s="61" t="inlineStr">
+      <c r="C18" s="72" t="inlineStr">
         <is>
           <t>Direct → «Ваші фото класні! Але Google вас не показує — маю рішення»</t>
         </is>
       </c>
     </row>
     <row r="19" ht="26" customHeight="1">
-      <c r="B19" s="61" t="inlineStr">
+      <c r="B19" s="72" t="inlineStr">
         <is>
           <t>🌐 Є сайт</t>
         </is>
       </c>
-      <c r="C19" s="61" t="inlineStr">
+      <c r="C19" s="72" t="inlineStr">
         <is>
           <t>Відкрий їх сайт на телефоні при власнику. Мовчки. Нехай побачать самі.</t>
         </is>
@@ -33830,56 +33989,56 @@
     </row>
     <row r="20" ht="8" customHeight="1"/>
     <row r="21" ht="26" customHeight="1">
-      <c r="B21" s="62" t="inlineStr">
+      <c r="B21" s="73" t="inlineStr">
         <is>
           <t>СКРИПТ ПЕРШОГО КОНТАКТУ</t>
         </is>
       </c>
-      <c r="C21" s="56" t="n"/>
+      <c r="C21" s="67" t="n"/>
     </row>
     <row r="22" ht="26" customHeight="1">
-      <c r="B22" s="63" t="inlineStr">
+      <c r="B22" s="74" t="inlineStr">
         <is>
           <t>Крок 1</t>
         </is>
       </c>
-      <c r="C22" s="63" t="inlineStr">
+      <c r="C22" s="74" t="inlineStr">
         <is>
           <t>«Добрий день! Я [ім'я], роблю сайти для кав'ярень у Львові»</t>
         </is>
       </c>
     </row>
     <row r="23" ht="26" customHeight="1">
-      <c r="B23" s="63" t="inlineStr">
+      <c r="B23" s="74" t="inlineStr">
         <is>
           <t>Крок 2</t>
         </is>
       </c>
-      <c r="C23" s="63" t="inlineStr">
+      <c r="C23" s="74" t="inlineStr">
         <is>
           <t>«Помітив що [ПРИЧИНА]. Хочу показати щось за 3 хвилини — можна?»</t>
         </is>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
-      <c r="B24" s="63" t="inlineStr">
+      <c r="B24" s="74" t="inlineStr">
         <is>
           <t>Крок 3</t>
         </is>
       </c>
-      <c r="C24" s="63" t="inlineStr">
+      <c r="C24" s="74" t="inlineStr">
         <is>
           <t>Показуєш liberty-cafe.onrender.com на своєму телефоні</t>
         </is>
       </c>
     </row>
     <row r="25" ht="26" customHeight="1">
-      <c r="B25" s="63" t="inlineStr">
+      <c r="B25" s="74" t="inlineStr">
         <is>
           <t>Крок 4</t>
         </is>
       </c>
-      <c r="C25" s="63" t="inlineStr">
+      <c r="C25" s="74" t="inlineStr">
         <is>
           <t>«Це я зроблю для вас за [ціна] і [строк]»</t>
         </is>
@@ -33887,56 +34046,56 @@
     </row>
     <row r="26" ht="8" customHeight="1"/>
     <row r="27" ht="26" customHeight="1">
-      <c r="B27" s="64" t="inlineStr">
+      <c r="B27" s="75" t="inlineStr">
         <is>
           <t>ЗАПЕРЕЧЕННЯ</t>
         </is>
       </c>
-      <c r="C27" s="56" t="n"/>
+      <c r="C27" s="67" t="n"/>
     </row>
     <row r="28" ht="26" customHeight="1">
-      <c r="B28" s="65" t="inlineStr">
+      <c r="B28" s="76" t="inlineStr">
         <is>
           <t>«Вже є Instagram»</t>
         </is>
       </c>
-      <c r="C28" s="65" t="inlineStr">
+      <c r="C28" s="76" t="inlineStr">
         <is>
           <t>«Instagram не індексується Google. Хто шукає 'кав'ярня Львів' — вас не знайде»</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
-      <c r="B29" s="65" t="inlineStr">
+      <c r="B29" s="76" t="inlineStr">
         <is>
           <t>«Немає часу»</t>
         </is>
       </c>
-      <c r="C29" s="65" t="inlineStr">
+      <c r="C29" s="76" t="inlineStr">
         <is>
           <t>«Від вас — 30 хв на початку. Далі самі оновлюєте за 2 кліки»</t>
         </is>
       </c>
     </row>
     <row r="30" ht="26" customHeight="1">
-      <c r="B30" s="65" t="inlineStr">
+      <c r="B30" s="76" t="inlineStr">
         <is>
           <t>«Дорого»</t>
         </is>
       </c>
-      <c r="C30" s="65" t="inlineStr">
+      <c r="C30" s="76" t="inlineStr">
         <is>
           <t>«Один новий клієнт з Google окупить сайт. Скільки у вас людей на день?»</t>
         </is>
       </c>
     </row>
     <row r="31" ht="26" customHeight="1">
-      <c r="B31" s="65" t="inlineStr">
+      <c r="B31" s="76" t="inlineStr">
         <is>
           <t>«Подумаю»</t>
         </is>
       </c>
-      <c r="C31" s="65" t="inlineStr">
+      <c r="C31" s="76" t="inlineStr">
         <is>
           <t>«Добре! Залишу демо — покажете партнеру?» → пиши через 3 дні</t>
         </is>

</xml_diff>